<commit_message>
Update RAG, README and test cases; remove report files
</commit_message>
<xml_diff>
--- a/Testcase.xlsx
+++ b/Testcase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Open_University\HK9_2025_2026\DO_AN\Training_system_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BCC6CB-8D1E-4076-89D8-CF4366EA3027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA66E4FB-E504-4B01-A83E-8C68C86F000B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="252" windowWidth="23256" windowHeight="12816" tabRatio="821" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="252" windowWidth="23256" windowHeight="12816" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -1904,7 +1904,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2165,9 +2165,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2188,9 +2185,6 @@
     </xf>
     <xf numFmtId="167" fontId="18" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2566,11 +2560,11 @@
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="107" t="s">
+      <c r="C6" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="108"/>
-      <c r="E6" s="109"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="107"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
@@ -2579,11 +2573,11 @@
       <c r="B7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="107" t="s">
+      <c r="C7" s="105" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="108"/>
-      <c r="E7" s="109"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="107"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
@@ -2797,12 +2791,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -2813,10 +2807,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -2830,54 +2824,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>300</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="158" t="s">
+      <c r="B5" s="156" t="s">
         <v>301</v>
       </c>
-      <c r="C5" s="159"/>
-      <c r="D5" s="160"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="158"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -2898,9 +2892,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -2921,16 +2915,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -2941,76 +2935,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="155" t="s">
+      <c r="A12" s="153" t="s">
         <v>302</v>
       </c>
-      <c r="B12" s="156"/>
-      <c r="C12" s="156"/>
-      <c r="D12" s="156"/>
-      <c r="E12" s="156"/>
-      <c r="F12" s="156"/>
-      <c r="G12" s="156"/>
-      <c r="H12" s="156"/>
-      <c r="I12" s="156"/>
-      <c r="J12" s="156"/>
-      <c r="K12" s="157"/>
+      <c r="B12" s="154"/>
+      <c r="C12" s="154"/>
+      <c r="D12" s="154"/>
+      <c r="E12" s="154"/>
+      <c r="F12" s="154"/>
+      <c r="G12" s="154"/>
+      <c r="H12" s="154"/>
+      <c r="I12" s="154"/>
+      <c r="J12" s="154"/>
+      <c r="K12" s="155"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -3022,11 +3016,11 @@
       <c r="C13" s="78" t="s">
         <v>305</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>306</v>
       </c>
-      <c r="E13" s="153"/>
-      <c r="F13" s="153"/>
+      <c r="E13" s="151"/>
+      <c r="F13" s="151"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -3040,7 +3034,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>307</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -3049,22 +3043,22 @@
       <c r="C14" s="78" t="s">
         <v>309</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>310</v>
       </c>
-      <c r="E14" s="153"/>
-      <c r="F14" s="153"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="105">
+      <c r="I14" s="104">
         <v>46268</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -3076,11 +3070,11 @@
       <c r="C15" s="78" t="s">
         <v>313</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>314</v>
       </c>
-      <c r="E15" s="153"/>
-      <c r="F15" s="153"/>
+      <c r="E15" s="151"/>
+      <c r="F15" s="151"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -3094,7 +3088,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>315</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -3103,22 +3097,22 @@
       <c r="C16" s="78" t="s">
         <v>317</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>318</v>
       </c>
-      <c r="E16" s="153"/>
-      <c r="F16" s="153"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="151"/>
+      <c r="F16" s="151"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="105">
+      <c r="I16" s="104">
         <v>46268</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101"/>
+      <c r="K16" s="100"/>
     </row>
     <row r="17" spans="1:11" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A17" s="76" t="s">
@@ -3130,11 +3124,11 @@
       <c r="C17" s="78" t="s">
         <v>321</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>322</v>
       </c>
-      <c r="E17" s="153"/>
-      <c r="F17" s="153"/>
+      <c r="E17" s="151"/>
+      <c r="F17" s="151"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -3157,11 +3151,11 @@
       <c r="C18" s="78" t="s">
         <v>325</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>326</v>
       </c>
-      <c r="E18" s="153"/>
-      <c r="F18" s="153"/>
+      <c r="E18" s="151"/>
+      <c r="F18" s="151"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -3178,9 +3172,9 @@
       <c r="A19" s="80"/>
       <c r="B19" s="81"/>
       <c r="C19" s="82"/>
-      <c r="D19" s="118"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
+      <c r="D19" s="116"/>
+      <c r="E19" s="138"/>
+      <c r="F19" s="138"/>
       <c r="G19" s="81"/>
       <c r="H19" s="81"/>
       <c r="I19" s="85"/>
@@ -3191,9 +3185,9 @@
       <c r="A20" s="80"/>
       <c r="B20" s="81"/>
       <c r="C20" s="82"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="140"/>
-      <c r="F20" s="140"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="138"/>
+      <c r="F20" s="138"/>
       <c r="G20" s="81"/>
       <c r="H20" s="81"/>
       <c r="I20" s="85"/>
@@ -3284,6 +3278,14 @@
     <mergeCell ref="D16:F16"/>
     <mergeCell ref="C9:C10"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{AFB9453E-E16B-41C8-88BE-6CE2960F79F8}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{6282D0F4-E2EC-440D-80F9-B1C595AC9810}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{6F1625DF-9C1E-4F8E-8BD6-41B947798885}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{4BDC002D-63A5-494B-AA48-B0E378322B57}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{B03FB5E0-8D8C-4CEF-A567-0BD9EF18E217}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{E937FE6A-6B14-4B75-BF94-6664B45F6D00}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3308,12 +3310,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -3324,10 +3326,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -3341,54 +3343,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>327</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>328</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -3409,9 +3411,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -3432,16 +3434,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -3452,76 +3454,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>329</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -3533,11 +3535,11 @@
       <c r="C13" s="78" t="s">
         <v>332</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>333</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -3551,7 +3553,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>334</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -3560,22 +3562,22 @@
       <c r="C14" s="78" t="s">
         <v>336</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>337</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="106" t="s">
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <v>46268</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -3587,11 +3589,11 @@
       <c r="C15" s="78" t="s">
         <v>340</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>341</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -3605,7 +3607,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>342</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -3614,22 +3616,22 @@
       <c r="C16" s="78" t="s">
         <v>344</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>345</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
-      <c r="H16" s="106" t="s">
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
+      <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <v>46268</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101"/>
+      <c r="K16" s="100"/>
     </row>
     <row r="17" spans="1:11" s="75" customFormat="1" ht="90" outlineLevel="1">
       <c r="A17" s="76" t="s">
@@ -3641,11 +3643,11 @@
       <c r="C17" s="78" t="s">
         <v>348</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>349</v>
       </c>
-      <c r="E17" s="153"/>
-      <c r="F17" s="153"/>
+      <c r="E17" s="151"/>
+      <c r="F17" s="151"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -3662,9 +3664,9 @@
       <c r="A18" s="80"/>
       <c r="B18" s="81"/>
       <c r="C18" s="82"/>
-      <c r="D18" s="118"/>
-      <c r="E18" s="140"/>
-      <c r="F18" s="140"/>
+      <c r="D18" s="116"/>
+      <c r="E18" s="138"/>
+      <c r="F18" s="138"/>
       <c r="G18" s="81"/>
       <c r="H18" s="81"/>
       <c r="I18" s="85"/>
@@ -3675,9 +3677,9 @@
       <c r="A19" s="80"/>
       <c r="B19" s="81"/>
       <c r="C19" s="82"/>
-      <c r="D19" s="118"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
+      <c r="D19" s="116"/>
+      <c r="E19" s="138"/>
+      <c r="F19" s="138"/>
       <c r="G19" s="81"/>
       <c r="H19" s="81"/>
       <c r="I19" s="85"/>
@@ -3688,9 +3690,9 @@
       <c r="A20" s="80"/>
       <c r="B20" s="81"/>
       <c r="C20" s="82"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="140"/>
-      <c r="F20" s="140"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="138"/>
+      <c r="F20" s="138"/>
       <c r="G20" s="81"/>
       <c r="H20" s="81"/>
       <c r="I20" s="85"/>
@@ -3701,9 +3703,9 @@
       <c r="A21" s="80"/>
       <c r="B21" s="81"/>
       <c r="C21" s="82"/>
-      <c r="D21" s="118"/>
-      <c r="E21" s="140"/>
-      <c r="F21" s="140"/>
+      <c r="D21" s="116"/>
+      <c r="E21" s="138"/>
+      <c r="F21" s="138"/>
       <c r="G21" s="81"/>
       <c r="H21" s="81"/>
       <c r="I21" s="85"/>
@@ -3795,6 +3797,13 @@
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="D14:F14"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{7A853944-0F60-4E84-9A41-9A6BF3639C10}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{C1177AE4-95DC-4CB5-AB82-16B0500B961C}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{CC0388A8-348C-4689-8FD8-40DF323EB8B8}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{F84AA5EC-5DD4-48B4-9E9C-C0F5E6217688}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{147D9DA5-DB76-431D-A86A-9CD7AD00D36B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -4245,12 +4254,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="60"/>
       <c r="F1" s="60"/>
       <c r="G1" s="61"/>
@@ -4261,10 +4270,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="134"/>
-      <c r="B2" s="134"/>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
+      <c r="A2" s="132"/>
+      <c r="B2" s="132"/>
+      <c r="C2" s="132"/>
+      <c r="D2" s="132"/>
       <c r="E2" s="60"/>
       <c r="F2" s="60"/>
       <c r="G2" s="61"/>
@@ -4278,54 +4287,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="108"/>
-      <c r="D3" s="109"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="107"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="116"/>
-      <c r="D4" s="122"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="120"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="116"/>
-      <c r="D5" s="122"/>
+      <c r="C5" s="114"/>
+      <c r="D5" s="120"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -4347,9 +4356,9 @@
       <c r="F6" s="60"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -4370,16 +4379,16 @@
       <c r="F7" s="72"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="108"/>
-      <c r="C8" s="108"/>
-      <c r="D8" s="108"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="106"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="106"/>
       <c r="E8" s="60"/>
       <c r="F8" s="60"/>
       <c r="G8" s="64"/>
@@ -4390,76 +4399,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="126"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="124"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="114"/>
-      <c r="B10" s="114"/>
-      <c r="C10" s="114"/>
-      <c r="D10" s="127"/>
-      <c r="E10" s="128"/>
-      <c r="F10" s="128"/>
-      <c r="G10" s="129"/>
-      <c r="H10" s="114"/>
-      <c r="I10" s="114"/>
-      <c r="J10" s="114"/>
-      <c r="K10" s="114"/>
+      <c r="A10" s="112"/>
+      <c r="B10" s="112"/>
+      <c r="C10" s="112"/>
+      <c r="D10" s="125"/>
+      <c r="E10" s="126"/>
+      <c r="F10" s="126"/>
+      <c r="G10" s="127"/>
+      <c r="H10" s="112"/>
+      <c r="I10" s="112"/>
+      <c r="J10" s="112"/>
+      <c r="K10" s="112"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="116"/>
-      <c r="C11" s="116"/>
-      <c r="D11" s="116"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="116"/>
-      <c r="G11" s="116"/>
-      <c r="H11" s="116"/>
-      <c r="I11" s="116"/>
-      <c r="J11" s="116"/>
-      <c r="K11" s="117"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="114"/>
+      <c r="J11" s="114"/>
+      <c r="K11" s="115"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="116"/>
-      <c r="C12" s="116"/>
-      <c r="D12" s="116"/>
-      <c r="E12" s="116"/>
-      <c r="F12" s="116"/>
-      <c r="G12" s="116"/>
-      <c r="H12" s="116"/>
-      <c r="I12" s="116"/>
-      <c r="J12" s="116"/>
-      <c r="K12" s="117"/>
+      <c r="B12" s="114"/>
+      <c r="C12" s="114"/>
+      <c r="D12" s="114"/>
+      <c r="E12" s="114"/>
+      <c r="F12" s="114"/>
+      <c r="G12" s="114"/>
+      <c r="H12" s="114"/>
+      <c r="I12" s="114"/>
+      <c r="J12" s="114"/>
+      <c r="K12" s="115"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="120" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -4471,13 +4480,13 @@
       <c r="C13" s="78" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="110" t="s">
+      <c r="D13" s="108" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="111"/>
-      <c r="F13" s="112"/>
+      <c r="E13" s="109"/>
+      <c r="F13" s="110"/>
       <c r="G13" s="77"/>
-      <c r="H13" s="99" t="s">
+      <c r="H13" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I13" s="79">
@@ -4498,13 +4507,13 @@
       <c r="C14" s="78" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="124" t="s">
+      <c r="D14" s="122" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="116"/>
-      <c r="F14" s="117"/>
+      <c r="E14" s="114"/>
+      <c r="F14" s="115"/>
       <c r="G14" s="77"/>
-      <c r="H14" s="99" t="s">
+      <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I14" s="79">
@@ -4525,13 +4534,13 @@
       <c r="C15" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="116"/>
-      <c r="F15" s="117"/>
+      <c r="E15" s="114"/>
+      <c r="F15" s="115"/>
       <c r="G15" s="77"/>
-      <c r="H15" s="99" t="s">
+      <c r="H15" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I15" s="79">
@@ -4552,13 +4561,13 @@
       <c r="C16" s="78" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="124" t="s">
+      <c r="D16" s="122" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="116"/>
-      <c r="F16" s="117"/>
+      <c r="E16" s="114"/>
+      <c r="F16" s="115"/>
       <c r="G16" s="77"/>
-      <c r="H16" s="99" t="s">
+      <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I16" s="79">
@@ -4579,13 +4588,13 @@
       <c r="C17" s="78" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="116"/>
-      <c r="F17" s="117"/>
+      <c r="E17" s="114"/>
+      <c r="F17" s="115"/>
       <c r="G17" s="77"/>
-      <c r="H17" s="99" t="s">
+      <c r="H17" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I17" s="79" t="s">
@@ -4608,13 +4617,13 @@
       <c r="C18" s="78" t="s">
         <v>62</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>63</v>
       </c>
-      <c r="E18" s="116"/>
-      <c r="F18" s="117"/>
+      <c r="E18" s="114"/>
+      <c r="F18" s="115"/>
       <c r="G18" s="77"/>
-      <c r="H18" s="99" t="s">
+      <c r="H18" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I18" s="79">
@@ -4629,9 +4638,9 @@
       <c r="A19" s="80"/>
       <c r="B19" s="81"/>
       <c r="C19" s="82"/>
-      <c r="D19" s="118"/>
-      <c r="E19" s="119"/>
-      <c r="F19" s="119"/>
+      <c r="D19" s="116"/>
+      <c r="E19" s="117"/>
+      <c r="F19" s="117"/>
       <c r="G19" s="81"/>
       <c r="H19" s="81"/>
       <c r="I19" s="85"/>
@@ -4642,9 +4651,9 @@
       <c r="A20" s="80"/>
       <c r="B20" s="81"/>
       <c r="C20" s="82"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
       <c r="G20" s="81"/>
       <c r="H20" s="81"/>
       <c r="I20" s="85"/>
@@ -4655,9 +4664,9 @@
       <c r="A21" s="80"/>
       <c r="B21" s="81"/>
       <c r="C21" s="82"/>
-      <c r="D21" s="118"/>
-      <c r="E21" s="119"/>
-      <c r="F21" s="119"/>
+      <c r="D21" s="116"/>
+      <c r="E21" s="117"/>
+      <c r="F21" s="117"/>
       <c r="G21" s="81"/>
       <c r="H21" s="81"/>
       <c r="I21" s="85"/>
@@ -4668,9 +4677,9 @@
       <c r="A22" s="80"/>
       <c r="B22" s="81"/>
       <c r="C22" s="82"/>
-      <c r="D22" s="118"/>
-      <c r="E22" s="119"/>
-      <c r="F22" s="119"/>
+      <c r="D22" s="116"/>
+      <c r="E22" s="117"/>
+      <c r="F22" s="117"/>
       <c r="G22" s="81"/>
       <c r="H22" s="81"/>
       <c r="I22" s="85"/>
@@ -4681,9 +4690,9 @@
       <c r="A23" s="80"/>
       <c r="B23" s="81"/>
       <c r="C23" s="82"/>
-      <c r="D23" s="118"/>
-      <c r="E23" s="119"/>
-      <c r="F23" s="119"/>
+      <c r="D23" s="116"/>
+      <c r="E23" s="117"/>
+      <c r="F23" s="117"/>
       <c r="G23" s="81"/>
       <c r="H23" s="81"/>
       <c r="I23" s="85"/>
@@ -4694,9 +4703,9 @@
       <c r="A24" s="80"/>
       <c r="B24" s="81"/>
       <c r="C24" s="82"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
+      <c r="D24" s="116"/>
+      <c r="E24" s="117"/>
+      <c r="F24" s="117"/>
       <c r="G24" s="81"/>
       <c r="H24" s="81"/>
       <c r="I24" s="85"/>
@@ -4818,12 +4827,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -4834,10 +4843,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -4851,54 +4860,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -4919,9 +4928,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -4942,16 +4951,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -4962,76 +4971,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -5043,11 +5052,11 @@
       <c r="C13" s="78" t="s">
         <v>364</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>365</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -5070,11 +5079,11 @@
       <c r="C14" s="78" t="s">
         <v>71</v>
       </c>
-      <c r="D14" s="124" t="s">
+      <c r="D14" s="122" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
       <c r="G14" s="77"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
@@ -5097,11 +5106,11 @@
       <c r="C15" s="78" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -5124,11 +5133,11 @@
       <c r="C16" s="78" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="124" t="s">
+      <c r="D16" s="122" t="s">
         <v>80</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
       <c r="G16" s="77"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
@@ -5151,11 +5160,11 @@
       <c r="C17" s="78" t="s">
         <v>83</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>84</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -5180,11 +5189,11 @@
       <c r="C18" s="78" t="s">
         <v>367</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>87</v>
       </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -5207,11 +5216,11 @@
       <c r="C19" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="D19" s="124" t="s">
+      <c r="D19" s="122" t="s">
         <v>91</v>
       </c>
-      <c r="E19" s="141"/>
-      <c r="F19" s="141"/>
+      <c r="E19" s="139"/>
+      <c r="F19" s="139"/>
       <c r="G19" s="77"/>
       <c r="H19" s="98" t="s">
         <v>361</v>
@@ -5234,11 +5243,11 @@
       <c r="C20" s="78" t="s">
         <v>94</v>
       </c>
-      <c r="D20" s="124" t="s">
+      <c r="D20" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="E20" s="141"/>
-      <c r="F20" s="141"/>
+      <c r="E20" s="139"/>
+      <c r="F20" s="139"/>
       <c r="G20" s="77"/>
       <c r="H20" s="98" t="s">
         <v>361</v>
@@ -5261,11 +5270,11 @@
       <c r="C21" s="78" t="s">
         <v>98</v>
       </c>
-      <c r="D21" s="124" t="s">
+      <c r="D21" s="122" t="s">
         <v>368</v>
       </c>
-      <c r="E21" s="141"/>
-      <c r="F21" s="141"/>
+      <c r="E21" s="139"/>
+      <c r="F21" s="139"/>
       <c r="G21" s="77"/>
       <c r="H21" s="98" t="s">
         <v>361</v>
@@ -5282,9 +5291,9 @@
       <c r="A22" s="80"/>
       <c r="B22" s="81"/>
       <c r="C22" s="82"/>
-      <c r="D22" s="118"/>
-      <c r="E22" s="119"/>
-      <c r="F22" s="119"/>
+      <c r="D22" s="116"/>
+      <c r="E22" s="117"/>
+      <c r="F22" s="117"/>
       <c r="G22" s="81"/>
       <c r="H22" s="81"/>
       <c r="I22" s="85"/>
@@ -5295,9 +5304,9 @@
       <c r="A23" s="80"/>
       <c r="B23" s="81"/>
       <c r="C23" s="82"/>
-      <c r="D23" s="118"/>
-      <c r="E23" s="119"/>
-      <c r="F23" s="119"/>
+      <c r="D23" s="116"/>
+      <c r="E23" s="117"/>
+      <c r="F23" s="117"/>
       <c r="G23" s="81"/>
       <c r="H23" s="81"/>
       <c r="I23" s="85"/>
@@ -5308,9 +5317,9 @@
       <c r="A24" s="80"/>
       <c r="B24" s="81"/>
       <c r="C24" s="82"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
+      <c r="D24" s="116"/>
+      <c r="E24" s="117"/>
+      <c r="F24" s="117"/>
       <c r="G24" s="81"/>
       <c r="H24" s="81"/>
       <c r="I24" s="85"/>
@@ -5321,9 +5330,9 @@
       <c r="A25" s="80"/>
       <c r="B25" s="81"/>
       <c r="C25" s="82"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="119"/>
-      <c r="F25" s="119"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="117"/>
+      <c r="F25" s="117"/>
       <c r="G25" s="81"/>
       <c r="H25" s="81"/>
       <c r="I25" s="85"/>
@@ -5334,9 +5343,9 @@
       <c r="A26" s="80"/>
       <c r="B26" s="81"/>
       <c r="C26" s="82"/>
-      <c r="D26" s="118"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="138"/>
+      <c r="F26" s="138"/>
       <c r="G26" s="81"/>
       <c r="H26" s="81"/>
       <c r="I26" s="85"/>
@@ -5418,8 +5427,19 @@
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="D23:F23"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{6D609119-452A-4AB4-9779-A145A65A7274}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{1107FC70-BBAF-477E-A2FD-07A685C6B67B}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{67FD90B7-E8DE-4AD7-876C-B6DF454D39FB}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{157F5D43-3BD6-480E-92F7-D7C0A48A28EC}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{B1BCD922-2BD9-4902-92C8-6F38D39ED89B}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{9F690D8F-4968-461A-863D-3618BB666460}"/>
+    <hyperlink ref="H19" r:id="rId7" xr:uid="{D13034E6-D968-4490-893E-C3959B1D311E}"/>
+    <hyperlink ref="H20" r:id="rId8" xr:uid="{FB0D2E99-FC71-4030-8655-365CDED7B15A}"/>
+    <hyperlink ref="H21" r:id="rId9" xr:uid="{96B3D6AF-F46C-4801-8A1D-AE2F9EAB4D51}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -5442,12 +5462,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -5458,10 +5478,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -5475,54 +5495,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>99</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>100</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -5543,9 +5563,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -5566,16 +5586,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -5586,76 +5606,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -5667,11 +5687,11 @@
       <c r="C13" s="78" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>369</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -5685,7 +5705,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>105</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -5694,22 +5714,22 @@
       <c r="C14" s="78" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>108</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <v>46267</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="105" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -5721,11 +5741,11 @@
       <c r="C15" s="78" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>112</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -5733,13 +5753,13 @@
       <c r="I15" s="79">
         <v>46267</v>
       </c>
-      <c r="J15" s="101" t="s">
+      <c r="J15" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>113</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -5748,22 +5768,22 @@
       <c r="C16" s="78" t="s">
         <v>115</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>116</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <v>46267</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101"/>
+      <c r="K16" s="100"/>
     </row>
     <row r="17" spans="1:11" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A17" s="76" t="s">
@@ -5775,11 +5795,11 @@
       <c r="C17" s="78" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>120</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -5787,7 +5807,7 @@
       <c r="I17" s="79">
         <v>46267</v>
       </c>
-      <c r="J17" s="101" t="s">
+      <c r="J17" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K17" s="78"/>
@@ -5802,11 +5822,11 @@
       <c r="C18" s="78" t="s">
         <v>123</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>124</v>
       </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -5814,7 +5834,7 @@
       <c r="I18" s="86">
         <v>46267</v>
       </c>
-      <c r="J18" s="101" t="s">
+      <c r="J18" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K18" s="78"/>
@@ -5829,11 +5849,11 @@
       <c r="C19" s="78" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="124" t="s">
+      <c r="D19" s="122" t="s">
         <v>128</v>
       </c>
-      <c r="E19" s="153"/>
-      <c r="F19" s="153"/>
+      <c r="E19" s="151"/>
+      <c r="F19" s="151"/>
       <c r="G19" s="77"/>
       <c r="H19" s="98" t="s">
         <v>361</v>
@@ -5841,7 +5861,7 @@
       <c r="I19" s="86">
         <v>46267</v>
       </c>
-      <c r="J19" s="101" t="s">
+      <c r="J19" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K19" s="78"/>
@@ -5856,11 +5876,11 @@
       <c r="C20" s="78" t="s">
         <v>131</v>
       </c>
-      <c r="D20" s="124" t="s">
+      <c r="D20" s="122" t="s">
         <v>132</v>
       </c>
-      <c r="E20" s="153"/>
-      <c r="F20" s="153"/>
+      <c r="E20" s="151"/>
+      <c r="F20" s="151"/>
       <c r="G20" s="77"/>
       <c r="H20" s="98" t="s">
         <v>361</v>
@@ -5868,7 +5888,7 @@
       <c r="I20" s="86">
         <v>46267</v>
       </c>
-      <c r="J20" s="101" t="s">
+      <c r="J20" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K20" s="78"/>
@@ -5883,11 +5903,11 @@
       <c r="C21" s="78" t="s">
         <v>370</v>
       </c>
-      <c r="D21" s="124" t="s">
+      <c r="D21" s="122" t="s">
         <v>371</v>
       </c>
-      <c r="E21" s="153"/>
-      <c r="F21" s="153"/>
+      <c r="E21" s="151"/>
+      <c r="F21" s="151"/>
       <c r="G21" s="77"/>
       <c r="H21" s="98" t="s">
         <v>361</v>
@@ -5895,7 +5915,7 @@
       <c r="I21" s="86">
         <v>46267</v>
       </c>
-      <c r="J21" s="101" t="s">
+      <c r="J21" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K21" s="78"/>
@@ -5910,11 +5930,11 @@
       <c r="C22" s="78" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="124" t="s">
+      <c r="D22" s="122" t="s">
         <v>138</v>
       </c>
-      <c r="E22" s="153"/>
-      <c r="F22" s="153"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="151"/>
       <c r="G22" s="77"/>
       <c r="H22" s="98" t="s">
         <v>361</v>
@@ -5922,7 +5942,7 @@
       <c r="I22" s="86">
         <v>46267</v>
       </c>
-      <c r="J22" s="101" t="s">
+      <c r="J22" s="100" t="s">
         <v>360</v>
       </c>
       <c r="K22" s="78"/>
@@ -5931,9 +5951,9 @@
       <c r="A23" s="80"/>
       <c r="B23" s="81"/>
       <c r="C23" s="82"/>
-      <c r="D23" s="118"/>
-      <c r="E23" s="140"/>
-      <c r="F23" s="140"/>
+      <c r="D23" s="116"/>
+      <c r="E23" s="138"/>
+      <c r="F23" s="138"/>
       <c r="G23" s="81"/>
       <c r="H23" s="81"/>
       <c r="I23" s="85"/>
@@ -5944,9 +5964,9 @@
       <c r="A24" s="80"/>
       <c r="B24" s="81"/>
       <c r="C24" s="82"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="140"/>
-      <c r="F24" s="140"/>
+      <c r="D24" s="116"/>
+      <c r="E24" s="138"/>
+      <c r="F24" s="138"/>
       <c r="G24" s="81"/>
       <c r="H24" s="81"/>
       <c r="I24" s="85"/>
@@ -5957,9 +5977,9 @@
       <c r="A25" s="80"/>
       <c r="B25" s="81"/>
       <c r="C25" s="82"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="140"/>
-      <c r="F25" s="140"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="138"/>
+      <c r="F25" s="138"/>
       <c r="G25" s="81"/>
       <c r="H25" s="81"/>
       <c r="I25" s="85"/>
@@ -5970,9 +5990,9 @@
       <c r="A26" s="80"/>
       <c r="B26" s="81"/>
       <c r="C26" s="82"/>
-      <c r="D26" s="118"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="138"/>
+      <c r="F26" s="138"/>
       <c r="G26" s="81"/>
       <c r="H26" s="81"/>
       <c r="I26" s="85"/>
@@ -5983,9 +6003,9 @@
       <c r="A27" s="80"/>
       <c r="B27" s="81"/>
       <c r="C27" s="82"/>
-      <c r="D27" s="118"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
+      <c r="D27" s="116"/>
+      <c r="E27" s="138"/>
+      <c r="F27" s="138"/>
       <c r="G27" s="81"/>
       <c r="H27" s="81"/>
       <c r="I27" s="85"/>
@@ -5996,9 +6016,9 @@
       <c r="A28" s="80"/>
       <c r="B28" s="81"/>
       <c r="C28" s="82"/>
-      <c r="D28" s="118"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
+      <c r="D28" s="116"/>
+      <c r="E28" s="138"/>
+      <c r="F28" s="138"/>
       <c r="G28" s="81"/>
       <c r="H28" s="81"/>
       <c r="I28" s="85"/>
@@ -6076,6 +6096,18 @@
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="D21:F21"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{F99C6520-AD75-48ED-A7D7-AE4A85927AE5}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{8B82A96B-FA6A-416B-BBE6-F9B2BBA196F7}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{809B1481-1184-490B-A50E-5778EC7B51BC}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{BF29B411-7183-4624-8783-08BC86C78982}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{C0F6AE2A-F5CE-45E7-ABBA-3F2B3A82EE47}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{4F393896-8281-4931-A03D-775127AB330D}"/>
+    <hyperlink ref="H19" r:id="rId7" xr:uid="{FC57409A-3A99-48DF-A9D6-262E4412F8BF}"/>
+    <hyperlink ref="H20" r:id="rId8" xr:uid="{5B23A86C-8169-4924-A9AB-804791198B13}"/>
+    <hyperlink ref="H21" r:id="rId9" xr:uid="{99EBC8CD-7AC8-4214-A53C-86D83E731079}"/>
+    <hyperlink ref="H22" r:id="rId10" xr:uid="{6B0B6E84-F3C3-43BE-81EE-2082DF274BDF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -6100,12 +6132,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -6116,10 +6148,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -6133,54 +6165,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -6201,9 +6233,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -6224,16 +6256,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -6244,76 +6276,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>141</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -6325,11 +6357,11 @@
       <c r="C13" s="78" t="s">
         <v>144</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>145</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -6343,7 +6375,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>146</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -6352,22 +6384,22 @@
       <c r="C14" s="78" t="s">
         <v>148</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <v>46267</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>372</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -6379,11 +6411,11 @@
       <c r="C15" s="78" t="s">
         <v>152</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>153</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -6397,7 +6429,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>154</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -6406,22 +6438,22 @@
       <c r="C16" s="78" t="s">
         <v>363</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>156</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <v>46267</v>
       </c>
       <c r="J16" s="78" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101"/>
+      <c r="K16" s="100"/>
     </row>
     <row r="17" spans="1:11" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A17" s="76" t="s">
@@ -6433,11 +6465,11 @@
       <c r="C17" s="78" t="s">
         <v>159</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>160</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -6460,11 +6492,11 @@
       <c r="C18" s="78" t="s">
         <v>163</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>164</v>
       </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -6487,11 +6519,11 @@
       <c r="C19" s="78" t="s">
         <v>167</v>
       </c>
-      <c r="D19" s="124" t="s">
+      <c r="D19" s="122" t="s">
         <v>168</v>
       </c>
-      <c r="E19" s="153"/>
-      <c r="F19" s="153"/>
+      <c r="E19" s="151"/>
+      <c r="F19" s="151"/>
       <c r="G19" s="77"/>
       <c r="H19" s="98" t="s">
         <v>361</v>
@@ -6516,11 +6548,11 @@
       <c r="C20" s="78" t="s">
         <v>171</v>
       </c>
-      <c r="D20" s="124" t="s">
+      <c r="D20" s="122" t="s">
         <v>172</v>
       </c>
-      <c r="E20" s="153"/>
-      <c r="F20" s="153"/>
+      <c r="E20" s="151"/>
+      <c r="F20" s="151"/>
       <c r="G20" s="77"/>
       <c r="H20" s="98" t="s">
         <v>361</v>
@@ -6537,11 +6569,11 @@
       <c r="A21" s="80"/>
       <c r="B21" s="81"/>
       <c r="C21" s="82"/>
-      <c r="D21" s="118"/>
-      <c r="E21" s="140"/>
-      <c r="F21" s="140"/>
+      <c r="D21" s="116"/>
+      <c r="E21" s="138"/>
+      <c r="F21" s="138"/>
       <c r="G21" s="81"/>
-      <c r="H21" s="104"/>
+      <c r="H21" s="103"/>
       <c r="I21" s="85"/>
       <c r="J21" s="82"/>
       <c r="K21" s="82"/>
@@ -6550,9 +6582,9 @@
       <c r="A22" s="80"/>
       <c r="B22" s="81"/>
       <c r="C22" s="82"/>
-      <c r="D22" s="118"/>
-      <c r="E22" s="140"/>
-      <c r="F22" s="140"/>
+      <c r="D22" s="116"/>
+      <c r="E22" s="138"/>
+      <c r="F22" s="138"/>
       <c r="G22" s="81"/>
       <c r="H22" s="81"/>
       <c r="I22" s="85"/>
@@ -6563,9 +6595,9 @@
       <c r="A23" s="80"/>
       <c r="B23" s="81"/>
       <c r="C23" s="82"/>
-      <c r="D23" s="118"/>
-      <c r="E23" s="140"/>
-      <c r="F23" s="140"/>
+      <c r="D23" s="116"/>
+      <c r="E23" s="138"/>
+      <c r="F23" s="138"/>
       <c r="G23" s="81"/>
       <c r="H23" s="81"/>
       <c r="I23" s="85"/>
@@ -6576,9 +6608,9 @@
       <c r="A24" s="80"/>
       <c r="B24" s="81"/>
       <c r="C24" s="82"/>
-      <c r="D24" s="118"/>
-      <c r="E24" s="140"/>
-      <c r="F24" s="140"/>
+      <c r="D24" s="116"/>
+      <c r="E24" s="138"/>
+      <c r="F24" s="138"/>
       <c r="G24" s="81"/>
       <c r="H24" s="81"/>
       <c r="I24" s="85"/>
@@ -6589,9 +6621,9 @@
       <c r="A25" s="80"/>
       <c r="B25" s="81"/>
       <c r="C25" s="82"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="140"/>
-      <c r="F25" s="140"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="138"/>
+      <c r="F25" s="138"/>
       <c r="G25" s="81"/>
       <c r="H25" s="81"/>
       <c r="I25" s="85"/>
@@ -6602,9 +6634,9 @@
       <c r="A26" s="80"/>
       <c r="B26" s="81"/>
       <c r="C26" s="82"/>
-      <c r="D26" s="118"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="138"/>
+      <c r="F26" s="138"/>
       <c r="G26" s="81"/>
       <c r="H26" s="81"/>
       <c r="I26" s="85"/>
@@ -6615,9 +6647,9 @@
       <c r="A27" s="80"/>
       <c r="B27" s="81"/>
       <c r="C27" s="82"/>
-      <c r="D27" s="118"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
+      <c r="D27" s="116"/>
+      <c r="E27" s="138"/>
+      <c r="F27" s="138"/>
       <c r="G27" s="81"/>
       <c r="H27" s="81"/>
       <c r="I27" s="85"/>
@@ -6628,9 +6660,9 @@
       <c r="A28" s="80"/>
       <c r="B28" s="81"/>
       <c r="C28" s="82"/>
-      <c r="D28" s="118"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
+      <c r="D28" s="116"/>
+      <c r="E28" s="138"/>
+      <c r="F28" s="138"/>
       <c r="G28" s="81"/>
       <c r="H28" s="81"/>
       <c r="I28" s="85"/>
@@ -6708,6 +6740,16 @@
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="D21:F21"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{C26CD2D4-57E1-4CCB-A832-8659EE034641}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{FE1D7C07-222B-4C5F-B1E8-B13912EB2580}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{997A1AF4-29CB-4177-BFEA-E5CACE633142}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{905CB24F-3B12-4A87-8636-62E03B710B9C}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{6137892C-D98B-41BF-96C9-CD4B2481A35C}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{BDD70B38-C670-4D66-848E-21EA2566949C}"/>
+    <hyperlink ref="H19" r:id="rId7" xr:uid="{279D22D8-9F60-4743-B5CC-C2AAB485AB92}"/>
+    <hyperlink ref="H20" r:id="rId8" xr:uid="{D40BE2B0-321C-4B94-A955-2FC1D1D6CB76}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -6732,12 +6774,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -6748,10 +6790,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -6765,54 +6807,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>173</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>174</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -6833,9 +6875,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -6856,16 +6898,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -6876,76 +6918,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>175</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -6957,11 +6999,11 @@
       <c r="C13" s="78" t="s">
         <v>178</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>179</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -6975,7 +7017,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="105" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>180</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -6984,22 +7026,22 @@
       <c r="C14" s="78" t="s">
         <v>182</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>183</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103" t="s">
+      <c r="I14" s="102" t="s">
         <v>385</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101" t="s">
+      <c r="K14" s="100" t="s">
         <v>374</v>
       </c>
     </row>
@@ -7013,11 +7055,11 @@
       <c r="C15" s="78" t="s">
         <v>186</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>187</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -7031,7 +7073,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>188</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -7040,22 +7082,22 @@
       <c r="C16" s="78" t="s">
         <v>190</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>191</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <v>46267</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101"/>
+      <c r="K16" s="100"/>
     </row>
     <row r="17" spans="1:11" s="75" customFormat="1" ht="105" outlineLevel="1">
       <c r="A17" s="76" t="s">
@@ -7067,11 +7109,11 @@
       <c r="C17" s="78" t="s">
         <v>194</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>195</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -7096,11 +7138,11 @@
       <c r="C18" s="78" t="s">
         <v>198</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>199</v>
       </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -7123,11 +7165,11 @@
       <c r="C19" s="78" t="s">
         <v>202</v>
       </c>
-      <c r="D19" s="124" t="s">
+      <c r="D19" s="122" t="s">
         <v>203</v>
       </c>
-      <c r="E19" s="153"/>
-      <c r="F19" s="153"/>
+      <c r="E19" s="151"/>
+      <c r="F19" s="151"/>
       <c r="G19" s="77"/>
       <c r="H19" s="98" t="s">
         <v>361</v>
@@ -7152,11 +7194,11 @@
       <c r="C20" s="78" t="s">
         <v>206</v>
       </c>
-      <c r="D20" s="124" t="s">
+      <c r="D20" s="122" t="s">
         <v>207</v>
       </c>
-      <c r="E20" s="153"/>
-      <c r="F20" s="153"/>
+      <c r="E20" s="151"/>
+      <c r="F20" s="151"/>
       <c r="G20" s="77"/>
       <c r="H20" s="98" t="s">
         <v>361</v>
@@ -7181,11 +7223,11 @@
       <c r="C21" s="78" t="s">
         <v>210</v>
       </c>
-      <c r="D21" s="124" t="s">
+      <c r="D21" s="122" t="s">
         <v>211</v>
       </c>
-      <c r="E21" s="153"/>
-      <c r="F21" s="153"/>
+      <c r="E21" s="151"/>
+      <c r="F21" s="151"/>
       <c r="G21" s="77"/>
       <c r="H21" s="98" t="s">
         <v>361</v>
@@ -7208,11 +7250,11 @@
       <c r="C22" s="78" t="s">
         <v>214</v>
       </c>
-      <c r="D22" s="124" t="s">
+      <c r="D22" s="122" t="s">
         <v>215</v>
       </c>
-      <c r="E22" s="153"/>
-      <c r="F22" s="153"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="151"/>
       <c r="G22" s="77"/>
       <c r="H22" s="98" t="s">
         <v>361</v>
@@ -7235,11 +7277,11 @@
       <c r="C23" s="78" t="s">
         <v>218</v>
       </c>
-      <c r="D23" s="124" t="s">
+      <c r="D23" s="122" t="s">
         <v>219</v>
       </c>
-      <c r="E23" s="153"/>
-      <c r="F23" s="153"/>
+      <c r="E23" s="151"/>
+      <c r="F23" s="151"/>
       <c r="G23" s="77"/>
       <c r="H23" s="98" t="s">
         <v>361</v>
@@ -7262,11 +7304,11 @@
       <c r="C24" s="78" t="s">
         <v>222</v>
       </c>
-      <c r="D24" s="124" t="s">
+      <c r="D24" s="122" t="s">
         <v>223</v>
       </c>
-      <c r="E24" s="153"/>
-      <c r="F24" s="153"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="151"/>
       <c r="G24" s="77"/>
       <c r="H24" s="98" t="s">
         <v>361</v>
@@ -7283,9 +7325,9 @@
       <c r="A25" s="80"/>
       <c r="B25" s="81"/>
       <c r="C25" s="82"/>
-      <c r="D25" s="118"/>
-      <c r="E25" s="140"/>
-      <c r="F25" s="140"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="138"/>
+      <c r="F25" s="138"/>
       <c r="G25" s="81"/>
       <c r="H25" s="81"/>
       <c r="I25" s="85"/>
@@ -7296,9 +7338,9 @@
       <c r="A26" s="80"/>
       <c r="B26" s="81"/>
       <c r="C26" s="82"/>
-      <c r="D26" s="118"/>
-      <c r="E26" s="140"/>
-      <c r="F26" s="140"/>
+      <c r="D26" s="116"/>
+      <c r="E26" s="138"/>
+      <c r="F26" s="138"/>
       <c r="G26" s="81"/>
       <c r="H26" s="81"/>
       <c r="I26" s="85"/>
@@ -7309,9 +7351,9 @@
       <c r="A27" s="80"/>
       <c r="B27" s="81"/>
       <c r="C27" s="82"/>
-      <c r="D27" s="118"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
+      <c r="D27" s="116"/>
+      <c r="E27" s="138"/>
+      <c r="F27" s="138"/>
       <c r="G27" s="81"/>
       <c r="H27" s="81"/>
       <c r="I27" s="85"/>
@@ -7322,9 +7364,9 @@
       <c r="A28" s="80"/>
       <c r="B28" s="81"/>
       <c r="C28" s="82"/>
-      <c r="D28" s="118"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
+      <c r="D28" s="116"/>
+      <c r="E28" s="138"/>
+      <c r="F28" s="138"/>
       <c r="G28" s="81"/>
       <c r="H28" s="81"/>
       <c r="I28" s="85"/>
@@ -7335,9 +7377,9 @@
       <c r="A29" s="80"/>
       <c r="B29" s="81"/>
       <c r="C29" s="82"/>
-      <c r="D29" s="118"/>
-      <c r="E29" s="140"/>
-      <c r="F29" s="140"/>
+      <c r="D29" s="116"/>
+      <c r="E29" s="138"/>
+      <c r="F29" s="138"/>
       <c r="G29" s="81"/>
       <c r="H29" s="81"/>
       <c r="I29" s="85"/>
@@ -7348,9 +7390,9 @@
       <c r="A30" s="80"/>
       <c r="B30" s="81"/>
       <c r="C30" s="82"/>
-      <c r="D30" s="118"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="140"/>
+      <c r="D30" s="116"/>
+      <c r="E30" s="138"/>
+      <c r="F30" s="138"/>
       <c r="G30" s="81"/>
       <c r="H30" s="81"/>
       <c r="I30" s="85"/>
@@ -7424,6 +7466,20 @@
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="D17:F17"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{DCF95C38-3810-49DD-A694-6A1F2680E66F}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{B374919E-40A2-4AA4-885F-50F4B440B319}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{21223D81-36BF-4CC8-A762-F578E3E3F309}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{1F8F5D94-A92E-4BDA-B004-2E9BE0FBB1E5}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{A6736AA7-F6B8-470D-8732-9363EFEED5B4}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{EA4CB7F6-7FFE-4D13-93E7-5EE85C054F53}"/>
+    <hyperlink ref="H19" r:id="rId7" xr:uid="{AF1E5A2C-C3D1-40DA-A7C0-636EDC3B795C}"/>
+    <hyperlink ref="H20" r:id="rId8" xr:uid="{FFAB2D6C-CC02-4B95-B070-C03A376B26E6}"/>
+    <hyperlink ref="H21" r:id="rId9" xr:uid="{C4E53F2A-AFA7-4D71-AF57-600B347476C2}"/>
+    <hyperlink ref="H22" r:id="rId10" xr:uid="{15FE0260-65B0-4838-AF11-DB81F4FBD7C8}"/>
+    <hyperlink ref="H23" r:id="rId11" xr:uid="{19812E23-C365-4190-A6DC-A9B696C13117}"/>
+    <hyperlink ref="H24" r:id="rId12" xr:uid="{6AF82603-E117-42C9-B4D8-C7229BDFF2FB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -7448,12 +7504,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -7464,10 +7520,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -7481,54 +7537,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>224</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>225</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -7549,9 +7605,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -7572,16 +7628,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -7592,76 +7648,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>226</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -7673,11 +7729,11 @@
       <c r="C13" s="78" t="s">
         <v>229</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>230</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -7691,7 +7747,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>231</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -7700,22 +7756,22 @@
       <c r="C14" s="78" t="s">
         <v>233</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>234</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <v>46267</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -7727,11 +7783,11 @@
       <c r="C15" s="78" t="s">
         <v>237</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>238</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -7745,7 +7801,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>239</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -7754,22 +7810,22 @@
       <c r="C16" s="78" t="s">
         <v>241</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>242</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <v>46267</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101" t="s">
+      <c r="K16" s="100" t="s">
         <v>378</v>
       </c>
     </row>
@@ -7783,11 +7839,11 @@
       <c r="C17" s="78" t="s">
         <v>245</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>246</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -7810,11 +7866,11 @@
       <c r="C18" s="78" t="s">
         <v>249</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>250</v>
       </c>
-      <c r="E18" s="153"/>
-      <c r="F18" s="153"/>
+      <c r="E18" s="151"/>
+      <c r="F18" s="151"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -7833,11 +7889,11 @@
       <c r="A19" s="80"/>
       <c r="B19" s="81"/>
       <c r="C19" s="82"/>
-      <c r="D19" s="118"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
+      <c r="D19" s="116"/>
+      <c r="E19" s="138"/>
+      <c r="F19" s="138"/>
       <c r="G19" s="81"/>
-      <c r="H19" s="104"/>
+      <c r="H19" s="103"/>
       <c r="I19" s="85"/>
       <c r="J19" s="82"/>
       <c r="K19" s="82"/>
@@ -7846,9 +7902,9 @@
       <c r="A20" s="80"/>
       <c r="B20" s="81"/>
       <c r="C20" s="82"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="140"/>
-      <c r="F20" s="140"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="138"/>
+      <c r="F20" s="138"/>
       <c r="G20" s="81"/>
       <c r="H20" s="81"/>
       <c r="I20" s="85"/>
@@ -7859,9 +7915,9 @@
       <c r="A21" s="80"/>
       <c r="B21" s="81"/>
       <c r="C21" s="82"/>
-      <c r="D21" s="118"/>
-      <c r="E21" s="140"/>
-      <c r="F21" s="140"/>
+      <c r="D21" s="116"/>
+      <c r="E21" s="138"/>
+      <c r="F21" s="138"/>
       <c r="G21" s="81"/>
       <c r="H21" s="81"/>
       <c r="I21" s="85"/>
@@ -7872,9 +7928,9 @@
       <c r="A22" s="80"/>
       <c r="B22" s="81"/>
       <c r="C22" s="82"/>
-      <c r="D22" s="118"/>
-      <c r="E22" s="140"/>
-      <c r="F22" s="140"/>
+      <c r="D22" s="116"/>
+      <c r="E22" s="138"/>
+      <c r="F22" s="138"/>
       <c r="G22" s="81"/>
       <c r="H22" s="81"/>
       <c r="I22" s="85"/>
@@ -7964,6 +8020,14 @@
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A9:A10"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{600A8603-8BE7-4381-9E32-81367C30EC33}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{9FBC0FAE-F733-472F-AA84-281073942FAC}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{55CFFB24-B10E-4591-8DBE-CF89F607F8FD}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{A35769B1-9651-4D63-9AAD-1D7732A8F859}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{70029CA1-0DBA-4E64-988B-0966299D1F1E}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{8C8D329F-C935-4BA8-8957-DF3A12DA1F36}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -7988,12 +8052,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -8004,10 +8068,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -8021,54 +8085,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>252</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -8089,9 +8153,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -8112,16 +8176,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -8132,76 +8196,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="123" t="s">
+      <c r="A12" s="121" t="s">
         <v>253</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="146"/>
+      <c r="B12" s="143"/>
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="143"/>
+      <c r="H12" s="143"/>
+      <c r="I12" s="143"/>
+      <c r="J12" s="143"/>
+      <c r="K12" s="144"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -8213,11 +8277,11 @@
       <c r="C13" s="78" t="s">
         <v>256</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>257</v>
       </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="146"/>
+      <c r="E13" s="143"/>
+      <c r="F13" s="144"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -8231,7 +8295,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="60" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>258</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -8240,22 +8304,22 @@
       <c r="C14" s="78" t="s">
         <v>260</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>261</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="146"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="143"/>
+      <c r="F14" s="144"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <v>46267</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="90" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -8267,11 +8331,11 @@
       <c r="C15" s="78" t="s">
         <v>264</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>265</v>
       </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="146"/>
+      <c r="E15" s="143"/>
+      <c r="F15" s="144"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -8285,7 +8349,7 @@
       <c r="K15" s="78"/>
     </row>
     <row r="16" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
-      <c r="A16" s="100" t="s">
+      <c r="A16" s="99" t="s">
         <v>266</v>
       </c>
       <c r="B16" s="77" t="s">
@@ -8294,22 +8358,22 @@
       <c r="C16" s="78" t="s">
         <v>268</v>
       </c>
-      <c r="D16" s="154" t="s">
+      <c r="D16" s="152" t="s">
         <v>269</v>
       </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="146"/>
-      <c r="G16" s="102"/>
+      <c r="E16" s="143"/>
+      <c r="F16" s="144"/>
+      <c r="G16" s="101"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
       </c>
-      <c r="I16" s="103" t="s">
+      <c r="I16" s="102" t="s">
         <v>383</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K16" s="101" t="s">
+      <c r="K16" s="100" t="s">
         <v>381</v>
       </c>
     </row>
@@ -8323,11 +8387,11 @@
       <c r="C17" s="78" t="s">
         <v>272</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>273</v>
       </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="146"/>
+      <c r="E17" s="143"/>
+      <c r="F17" s="144"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -8352,11 +8416,11 @@
       <c r="C18" s="78" t="s">
         <v>276</v>
       </c>
-      <c r="D18" s="124" t="s">
+      <c r="D18" s="122" t="s">
         <v>277</v>
       </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="146"/>
+      <c r="E18" s="143"/>
+      <c r="F18" s="144"/>
       <c r="G18" s="77"/>
       <c r="H18" s="98" t="s">
         <v>361</v>
@@ -8373,9 +8437,9 @@
       <c r="A19" s="80"/>
       <c r="B19" s="81"/>
       <c r="C19" s="82"/>
-      <c r="D19" s="118"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
+      <c r="D19" s="116"/>
+      <c r="E19" s="138"/>
+      <c r="F19" s="138"/>
       <c r="G19" s="81"/>
       <c r="H19" s="81"/>
       <c r="I19" s="85"/>
@@ -8386,9 +8450,9 @@
       <c r="A20" s="80"/>
       <c r="B20" s="81"/>
       <c r="C20" s="82"/>
-      <c r="D20" s="118"/>
-      <c r="E20" s="140"/>
-      <c r="F20" s="140"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="138"/>
+      <c r="F20" s="138"/>
       <c r="G20" s="81"/>
       <c r="H20" s="81"/>
       <c r="I20" s="85"/>
@@ -8482,6 +8546,14 @@
     <mergeCell ref="J9:J10"/>
     <mergeCell ref="A11:K11"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{15F51B9F-581C-4698-90A9-634D2662C6D1}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{F6A61621-8793-43DA-B79D-F5233F50F166}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{3E9F54AD-FEF6-43F1-BE97-FDE70A661EB3}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{012351B4-9898-4766-8A3F-64321AFC3845}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{2412E0D2-7DAD-4A35-BCA7-CE103D837D93}"/>
+    <hyperlink ref="H18" r:id="rId6" xr:uid="{BF766E84-3660-4EC8-ADFF-ACB5CC6B9868}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -8506,12 +8578,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="34" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="123"/>
+      <c r="D1" s="123"/>
       <c r="E1" s="61"/>
       <c r="F1" s="61"/>
       <c r="G1" s="61"/>
@@ -8522,10 +8594,10 @@
       <c r="L1" s="33"/>
     </row>
     <row r="2" spans="1:12" s="34" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
-      <c r="A2" s="152"/>
-      <c r="B2" s="152"/>
-      <c r="C2" s="152"/>
-      <c r="D2" s="152"/>
+      <c r="A2" s="150"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="61"/>
       <c r="F2" s="61"/>
       <c r="G2" s="61"/>
@@ -8539,54 +8611,54 @@
       <c r="A3" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="134" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="142"/>
-      <c r="D3" s="143"/>
+      <c r="C3" s="140"/>
+      <c r="D3" s="141"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
       <c r="L3" s="33"/>
     </row>
     <row r="4" spans="1:12" s="34" customFormat="1" ht="30">
       <c r="A4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="135" t="s">
+      <c r="B4" s="133" t="s">
         <v>278</v>
       </c>
-      <c r="C4" s="145"/>
-      <c r="D4" s="147"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="145"/>
       <c r="E4" s="63"/>
       <c r="F4" s="63"/>
       <c r="G4" s="63"/>
       <c r="H4" s="63"/>
-      <c r="I4" s="130"/>
-      <c r="J4" s="125"/>
-      <c r="K4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="123"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" s="68" customFormat="1" ht="26.25" customHeight="1">
       <c r="A5" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="119" t="s">
         <v>279</v>
       </c>
-      <c r="C5" s="145"/>
-      <c r="D5" s="147"/>
+      <c r="C5" s="143"/>
+      <c r="D5" s="145"/>
       <c r="E5" s="66"/>
       <c r="F5" s="66"/>
       <c r="G5" s="66"/>
       <c r="H5" s="66"/>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="132"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
       <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -8607,9 +8679,9 @@
       <c r="F6" s="64"/>
       <c r="G6" s="64"/>
       <c r="H6" s="64"/>
-      <c r="I6" s="130"/>
-      <c r="J6" s="125"/>
-      <c r="K6" s="125"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="123"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="33"/>
     </row>
     <row r="7" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
@@ -8630,16 +8702,16 @@
       <c r="F7" s="73"/>
       <c r="G7" s="73"/>
       <c r="H7" s="73"/>
-      <c r="I7" s="130"/>
-      <c r="J7" s="125"/>
-      <c r="K7" s="125"/>
+      <c r="I7" s="128"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="123"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" s="34" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="138"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
+      <c r="A8" s="136"/>
+      <c r="B8" s="140"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="64"/>
@@ -8650,76 +8722,76 @@
       <c r="L8" s="33"/>
     </row>
     <row r="9" spans="1:12" s="34" customFormat="1" ht="18" customHeight="1">
-      <c r="A9" s="113" t="s">
+      <c r="A9" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="120" t="s">
+      <c r="B9" s="118" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="113" t="s">
+      <c r="C9" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="113" t="s">
+      <c r="D9" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="148"/>
-      <c r="H9" s="113" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="146"/>
+      <c r="H9" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="137" t="s">
+      <c r="I9" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="137" t="s">
+      <c r="J9" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="137" t="s">
+      <c r="K9" s="135" t="s">
         <v>38</v>
       </c>
       <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" s="34" customFormat="1" ht="12" customHeight="1">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="150"/>
-      <c r="F10" s="150"/>
-      <c r="G10" s="151"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
-      <c r="K10" s="144"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="142"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="147"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="148"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="142"/>
+      <c r="I10" s="142"/>
+      <c r="J10" s="142"/>
+      <c r="K10" s="142"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
-      <c r="A11" s="115"/>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="146"/>
+      <c r="A11" s="113"/>
+      <c r="B11" s="143"/>
+      <c r="C11" s="143"/>
+      <c r="D11" s="143"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="143"/>
+      <c r="G11" s="143"/>
+      <c r="H11" s="143"/>
+      <c r="I11" s="143"/>
+      <c r="J11" s="143"/>
+      <c r="K11" s="144"/>
     </row>
     <row r="12" spans="1:12" s="75" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A12" s="155" t="s">
+      <c r="A12" s="153" t="s">
         <v>280</v>
       </c>
-      <c r="B12" s="156"/>
-      <c r="C12" s="156"/>
-      <c r="D12" s="156"/>
-      <c r="E12" s="156"/>
-      <c r="F12" s="156"/>
-      <c r="G12" s="156"/>
-      <c r="H12" s="156"/>
-      <c r="I12" s="156"/>
-      <c r="J12" s="156"/>
-      <c r="K12" s="157"/>
+      <c r="B12" s="154"/>
+      <c r="C12" s="154"/>
+      <c r="D12" s="154"/>
+      <c r="E12" s="154"/>
+      <c r="F12" s="154"/>
+      <c r="G12" s="154"/>
+      <c r="H12" s="154"/>
+      <c r="I12" s="154"/>
+      <c r="J12" s="154"/>
+      <c r="K12" s="155"/>
     </row>
     <row r="13" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A13" s="76" t="s">
@@ -8731,11 +8803,11 @@
       <c r="C13" s="78" t="s">
         <v>380</v>
       </c>
-      <c r="D13" s="124" t="s">
+      <c r="D13" s="122" t="s">
         <v>283</v>
       </c>
-      <c r="E13" s="153"/>
-      <c r="F13" s="153"/>
+      <c r="E13" s="151"/>
+      <c r="F13" s="151"/>
       <c r="G13" s="77"/>
       <c r="H13" s="98" t="s">
         <v>361</v>
@@ -8749,7 +8821,7 @@
       <c r="K13" s="78"/>
     </row>
     <row r="14" spans="1:12" s="75" customFormat="1" ht="45" outlineLevel="1">
-      <c r="A14" s="100" t="s">
+      <c r="A14" s="99" t="s">
         <v>284</v>
       </c>
       <c r="B14" s="77" t="s">
@@ -8758,22 +8830,22 @@
       <c r="C14" s="78" t="s">
         <v>286</v>
       </c>
-      <c r="D14" s="154" t="s">
+      <c r="D14" s="152" t="s">
         <v>287</v>
       </c>
-      <c r="E14" s="153"/>
-      <c r="F14" s="153"/>
-      <c r="G14" s="102"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="101"/>
       <c r="H14" s="98" t="s">
         <v>361</v>
       </c>
       <c r="I14" s="79">
         <v>46268</v>
       </c>
-      <c r="J14" s="101" t="s">
+      <c r="J14" s="100" t="s">
         <v>360</v>
       </c>
-      <c r="K14" s="101"/>
+      <c r="K14" s="100"/>
     </row>
     <row r="15" spans="1:12" s="75" customFormat="1" ht="75" outlineLevel="1">
       <c r="A15" s="76" t="s">
@@ -8785,11 +8857,11 @@
       <c r="C15" s="78" t="s">
         <v>290</v>
       </c>
-      <c r="D15" s="124" t="s">
+      <c r="D15" s="122" t="s">
         <v>291</v>
       </c>
-      <c r="E15" s="153"/>
-      <c r="F15" s="153"/>
+      <c r="E15" s="151"/>
+      <c r="F15" s="151"/>
       <c r="G15" s="77"/>
       <c r="H15" s="98" t="s">
         <v>361</v>
@@ -8812,11 +8884,11 @@
       <c r="C16" s="78" t="s">
         <v>295</v>
       </c>
-      <c r="D16" s="124" t="s">
+      <c r="D16" s="122" t="s">
         <v>296</v>
       </c>
-      <c r="E16" s="153"/>
-      <c r="F16" s="153"/>
+      <c r="E16" s="151"/>
+      <c r="F16" s="151"/>
       <c r="G16" s="77"/>
       <c r="H16" s="98" t="s">
         <v>361</v>
@@ -8839,11 +8911,11 @@
       <c r="C17" s="78" t="s">
         <v>298</v>
       </c>
-      <c r="D17" s="124" t="s">
+      <c r="D17" s="122" t="s">
         <v>299</v>
       </c>
-      <c r="E17" s="153"/>
-      <c r="F17" s="153"/>
+      <c r="E17" s="151"/>
+      <c r="F17" s="151"/>
       <c r="G17" s="77"/>
       <c r="H17" s="98" t="s">
         <v>361</v>
@@ -8860,9 +8932,9 @@
       <c r="A18" s="80"/>
       <c r="B18" s="81"/>
       <c r="C18" s="82"/>
-      <c r="D18" s="118"/>
-      <c r="E18" s="140"/>
-      <c r="F18" s="140"/>
+      <c r="D18" s="116"/>
+      <c r="E18" s="138"/>
+      <c r="F18" s="138"/>
       <c r="G18" s="81"/>
       <c r="H18" s="81"/>
       <c r="I18" s="85"/>
@@ -8954,6 +9026,13 @@
     <mergeCell ref="J9:J10"/>
     <mergeCell ref="A11:K11"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H13" r:id="rId1" xr:uid="{26A7495E-CBCC-4F67-9C6C-D54C5330A502}"/>
+    <hyperlink ref="H14" r:id="rId2" xr:uid="{63C508FF-955E-419A-8C81-F935C1144533}"/>
+    <hyperlink ref="H15" r:id="rId3" xr:uid="{D1D87319-6A8B-4543-8E04-F6895895CB6B}"/>
+    <hyperlink ref="H16" r:id="rId4" xr:uid="{89A97386-4025-4054-A725-04D8CE80DF0E}"/>
+    <hyperlink ref="H17" r:id="rId5" xr:uid="{38AC7179-0F12-4F81-9AE1-8D5CAC4705B8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>